<commit_message>
added steps, updated progress
</commit_message>
<xml_diff>
--- a/analysis_steps.xlsx
+++ b/analysis_steps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TestFolderSJ\mt_lion_crossings_and_corridors\mt_lion_crossings_and_corridors\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://egretorg-my.sharepoint.com/personal/scott_jennings_egret_org/Documents/Projects/other_research/mt_lion_crossings_and_corridors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6998644D-BCD5-4449-8257-06DBCE91F9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{6998644D-BCD5-4449-8257-06DBCE91F9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5D345CC-B35B-455A-81AE-7113515933C6}"/>
   <bookViews>
-    <workbookView xWindow="31020" yWindow="105" windowWidth="19515" windowHeight="12780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="0" windowWidth="19190" windowHeight="10320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
   <si>
     <t>notes</t>
   </si>
@@ -63,9 +63,6 @@
     <t>do UD look ok for big movement/dispersing lions?</t>
   </si>
   <si>
-    <t>any lions to exclude based on UD quirks?</t>
-  </si>
-  <si>
     <t>check naïve crossings for all lions with OK UD</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>how many crossings per lion</t>
   </si>
   <si>
-    <t>any lions to exclude for too few crossings? Might decide not to exclude any for this reason; double check used vs available</t>
-  </si>
-  <si>
     <t>extract segment habitat, etc. for segments in new UD</t>
   </si>
   <si>
@@ -127,6 +121,51 @@
   </si>
   <si>
     <t>sort out git commits/ignore between C and E</t>
+  </si>
+  <si>
+    <t>decided to fill holes</t>
+  </si>
+  <si>
+    <t>yup</t>
+  </si>
+  <si>
+    <t>any lions to exclude based on UD quirks? Yes, excluding P34 for quirky home range and few overall fixes/days tracked</t>
+  </si>
+  <si>
+    <t>all good except P30 who only had crossings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">any lions to exclude for too few crossings? The ratio of crossing steps to total steps is fairly similar between lions with few and lots of crossings, so might not to exclude any for this reason; double check used vs available. </t>
+  </si>
+  <si>
+    <t>get road segments for new UD</t>
+  </si>
+  <si>
+    <t>more lions = more area = more segments</t>
+  </si>
+  <si>
+    <t>get BBMM whole segments</t>
+  </si>
+  <si>
+    <t>this should be one segment per BBMM</t>
+  </si>
+  <si>
+    <t>tre+shr</t>
+  </si>
+  <si>
+    <t>impervious</t>
+  </si>
+  <si>
+    <t>calculate cohesion</t>
+  </si>
+  <si>
+    <t>riparian intersections</t>
+  </si>
+  <si>
+    <t>bridges</t>
+  </si>
+  <si>
+    <t>class</t>
   </si>
 </sst>
 </file>
@@ -142,7 +181,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -173,6 +212,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -186,15 +231,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,20 +519,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="54" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="54" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>5</v>
       </c>
       <c r="C1" t="s">
@@ -499,176 +543,279 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="5">
         <v>45895</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="7"/>
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="5">
+        <v>45896</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>34</v>
+      </c>
+      <c r="D4" s="5">
+        <v>45897</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
       </c>
+      <c r="D5" s="5">
+        <v>45897</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>8</v>
       </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="5">
+        <v>45897</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
       </c>
+      <c r="D7" s="5">
+        <v>45897</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
       </c>
+      <c r="D8" s="5">
+        <v>45897</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="5">
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="5">
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="5">
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="5">
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="5">
+        <v>45898</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="5">
+        <v>45899</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
+      <c r="B27" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="1" t="s">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="1" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="1" t="s">
+      <c r="B30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
         <v>30</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>